<commit_message>
updated all app forms fixed compile warnings (#186) (#156)
Co-authored-by: stephenmhuli <115163897+stephenmhuli@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/forms/app/postpartum.xlsx
+++ b/forms/app/postpartum.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1480" uniqueCount="806">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1488" uniqueCount="806">
   <si>
     <t>type</t>
   </si>
@@ -2727,15 +2727,15 @@
     </xf>
     <xf borderId="1" fillId="2" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="3" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
@@ -3925,7 +3925,7 @@
       <c r="A46" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B46" s="9" t="s">
+      <c r="B46" s="1" t="s">
         <v>92</v>
       </c>
       <c r="C46" s="1"/>
@@ -3937,7 +3937,7 @@
       <c r="I46" s="1"/>
       <c r="J46" s="1"/>
       <c r="K46" s="1"/>
-      <c r="L46" s="10" t="s">
+      <c r="L46" s="5" t="s">
         <v>93</v>
       </c>
       <c r="M46" s="1"/>
@@ -4029,7 +4029,7 @@
       <c r="C49" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="D49" s="11" t="s">
+      <c r="D49" s="9" t="s">
         <v>99</v>
       </c>
       <c r="E49" s="1"/>
@@ -4179,7 +4179,7 @@
       <c r="A57" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B57" s="12" t="s">
+      <c r="B57" s="10" t="s">
         <v>105</v>
       </c>
     </row>
@@ -4187,7 +4187,7 @@
       <c r="A58" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B58" s="12" t="s">
+      <c r="B58" s="10" t="s">
         <v>121</v>
       </c>
       <c r="C58" s="1" t="s">
@@ -4201,7 +4201,7 @@
       <c r="A59" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B59" s="12" t="s">
+      <c r="B59" s="10" t="s">
         <v>124</v>
       </c>
       <c r="C59" s="1" t="s">
@@ -4215,7 +4215,7 @@
       <c r="A60" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B60" s="12" t="s">
+      <c r="B60" s="10" t="s">
         <v>121</v>
       </c>
     </row>
@@ -4223,7 +4223,7 @@
       <c r="A61" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B61" s="12" t="s">
+      <c r="B61" s="10" t="s">
         <v>127</v>
       </c>
       <c r="C61" s="1" t="s">
@@ -4237,7 +4237,7 @@
       <c r="A62" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B62" s="12" t="s">
+      <c r="B62" s="10" t="s">
         <v>130</v>
       </c>
       <c r="C62" s="1" t="s">
@@ -4251,7 +4251,7 @@
       <c r="A63" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B63" s="12" t="s">
+      <c r="B63" s="10" t="s">
         <v>133</v>
       </c>
       <c r="C63" s="1" t="s">
@@ -4265,7 +4265,7 @@
       <c r="A64" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B64" s="12" t="s">
+      <c r="B64" s="10" t="s">
         <v>134</v>
       </c>
       <c r="C64" s="1" t="s">
@@ -4279,10 +4279,10 @@
       <c r="A65" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B65" s="12" t="s">
+      <c r="B65" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="C65" s="13" t="s">
+      <c r="C65" s="11" t="s">
         <v>138</v>
       </c>
       <c r="D65" s="1" t="s">
@@ -4294,7 +4294,7 @@
       <c r="A66" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B66" s="12" t="s">
+      <c r="B66" s="10" t="s">
         <v>140</v>
       </c>
       <c r="C66" s="1" t="s">
@@ -4308,7 +4308,7 @@
       <c r="A67" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="B67" s="12" t="s">
+      <c r="B67" s="10" t="s">
         <v>143</v>
       </c>
       <c r="C67" s="1" t="s">
@@ -4325,7 +4325,7 @@
       <c r="A68" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="B68" s="12" t="s">
+      <c r="B68" s="10" t="s">
         <v>147</v>
       </c>
       <c r="C68" s="1" t="s">
@@ -4342,7 +4342,7 @@
       <c r="A69" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="B69" s="12" t="s">
+      <c r="B69" s="10" t="s">
         <v>150</v>
       </c>
       <c r="C69" s="1" t="s">
@@ -4359,7 +4359,7 @@
       <c r="A70" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B70" s="12" t="s">
+      <c r="B70" s="10" t="s">
         <v>140</v>
       </c>
     </row>
@@ -4367,7 +4367,7 @@
       <c r="A71" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="B71" s="12" t="s">
+      <c r="B71" s="10" t="s">
         <v>153</v>
       </c>
       <c r="C71" s="1" t="s">
@@ -4387,7 +4387,7 @@
       <c r="A72" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B72" s="12" t="s">
+      <c r="B72" s="10" t="s">
         <v>157</v>
       </c>
       <c r="C72" s="1" t="s">
@@ -4404,7 +4404,7 @@
       <c r="A73" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B73" s="12" t="s">
+      <c r="B73" s="10" t="s">
         <v>161</v>
       </c>
       <c r="C73" s="1" t="s">
@@ -4421,7 +4421,7 @@
       <c r="A74" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B74" s="12" t="s">
+      <c r="B74" s="10" t="s">
         <v>133</v>
       </c>
     </row>
@@ -4429,7 +4429,7 @@
       <c r="A75" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B75" s="12" t="s">
+      <c r="B75" s="10" t="s">
         <v>127</v>
       </c>
       <c r="C75" s="1"/>
@@ -4440,7 +4440,7 @@
       <c r="A76" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B76" s="12" t="s">
+      <c r="B76" s="10" t="s">
         <v>165</v>
       </c>
       <c r="C76" s="1" t="s">
@@ -4460,7 +4460,7 @@
       <c r="A77" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B77" s="12" t="s">
+      <c r="B77" s="10" t="s">
         <v>169</v>
       </c>
       <c r="C77" s="1" t="s">
@@ -4474,7 +4474,7 @@
       <c r="A78" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B78" s="12" t="s">
+      <c r="B78" s="10" t="s">
         <v>172</v>
       </c>
       <c r="C78" s="1" t="s">
@@ -4488,7 +4488,7 @@
       <c r="A79" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="B79" s="12" t="s">
+      <c r="B79" s="10" t="s">
         <v>173</v>
       </c>
       <c r="C79" s="1" t="s">
@@ -4505,7 +4505,7 @@
       <c r="A80" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="B80" s="12" t="s">
+      <c r="B80" s="10" t="s">
         <v>176</v>
       </c>
       <c r="C80" s="1" t="s">
@@ -4522,7 +4522,7 @@
       <c r="A81" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="B81" s="12" t="s">
+      <c r="B81" s="10" t="s">
         <v>179</v>
       </c>
       <c r="C81" s="1" t="s">
@@ -4539,7 +4539,7 @@
       <c r="A82" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="B82" s="12" t="s">
+      <c r="B82" s="10" t="s">
         <v>182</v>
       </c>
       <c r="C82" s="1" t="s">
@@ -4556,7 +4556,7 @@
       <c r="A83" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="B83" s="12" t="s">
+      <c r="B83" s="10" t="s">
         <v>185</v>
       </c>
       <c r="C83" s="1" t="s">
@@ -4573,7 +4573,7 @@
       <c r="A84" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="B84" s="12" t="s">
+      <c r="B84" s="10" t="s">
         <v>188</v>
       </c>
       <c r="C84" s="1" t="s">
@@ -4590,7 +4590,7 @@
       <c r="A85" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="B85" s="12" t="s">
+      <c r="B85" s="10" t="s">
         <v>191</v>
       </c>
       <c r="C85" s="1" t="s">
@@ -4607,7 +4607,7 @@
       <c r="A86" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="B86" s="12" t="s">
+      <c r="B86" s="10" t="s">
         <v>194</v>
       </c>
       <c r="C86" s="1" t="s">
@@ -4624,7 +4624,7 @@
       <c r="A87" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="B87" s="12" t="s">
+      <c r="B87" s="10" t="s">
         <v>197</v>
       </c>
       <c r="C87" s="1" t="s">
@@ -4641,7 +4641,7 @@
       <c r="A88" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="B88" s="12" t="s">
+      <c r="B88" s="10" t="s">
         <v>200</v>
       </c>
       <c r="C88" s="1" t="s">
@@ -4658,7 +4658,7 @@
       <c r="A89" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="B89" s="12" t="s">
+      <c r="B89" s="10" t="s">
         <v>203</v>
       </c>
       <c r="C89" s="1" t="s">
@@ -4675,7 +4675,7 @@
       <c r="A90" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="B90" s="12" t="s">
+      <c r="B90" s="10" t="s">
         <v>206</v>
       </c>
       <c r="C90" s="1" t="s">
@@ -4692,7 +4692,7 @@
       <c r="A91" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="B91" s="12" t="s">
+      <c r="B91" s="10" t="s">
         <v>209</v>
       </c>
       <c r="C91" s="1" t="s">
@@ -4709,7 +4709,7 @@
       <c r="A92" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B92" s="12" t="s">
+      <c r="B92" s="10" t="s">
         <v>172</v>
       </c>
     </row>
@@ -4717,7 +4717,7 @@
       <c r="A93" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="B93" s="12" t="s">
+      <c r="B93" s="10" t="s">
         <v>213</v>
       </c>
       <c r="C93" s="1" t="s">
@@ -4737,7 +4737,7 @@
       <c r="A94" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="B94" s="12" t="s">
+      <c r="B94" s="10" t="s">
         <v>217</v>
       </c>
       <c r="C94" s="1" t="s">
@@ -4757,7 +4757,7 @@
       <c r="A95" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B95" s="12" t="s">
+      <c r="B95" s="10" t="s">
         <v>221</v>
       </c>
       <c r="C95" s="1" t="s">
@@ -4774,7 +4774,7 @@
       <c r="A96" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="B96" s="12" t="s">
+      <c r="B96" s="10" t="s">
         <v>225</v>
       </c>
       <c r="C96" s="1" t="s">
@@ -4794,7 +4794,7 @@
       <c r="A97" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B97" s="12" t="s">
+      <c r="B97" s="10" t="s">
         <v>228</v>
       </c>
       <c r="C97" s="1" t="s">
@@ -4811,7 +4811,7 @@
       <c r="A98" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B98" s="12" t="s">
+      <c r="B98" s="10" t="s">
         <v>232</v>
       </c>
       <c r="C98" s="1" t="s">
@@ -4828,7 +4828,7 @@
       <c r="A99" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B99" s="12" t="s">
+      <c r="B99" s="10" t="s">
         <v>236</v>
       </c>
       <c r="C99" s="1" t="s">
@@ -4845,7 +4845,7 @@
       <c r="A100" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B100" s="12" t="s">
+      <c r="B100" s="10" t="s">
         <v>165</v>
       </c>
     </row>
@@ -4853,7 +4853,7 @@
       <c r="A101" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B101" s="12" t="s">
+      <c r="B101" s="10" t="s">
         <v>240</v>
       </c>
       <c r="C101" s="1" t="s">
@@ -4874,7 +4874,7 @@
       <c r="A102" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B102" s="12" t="s">
+      <c r="B102" s="10" t="s">
         <v>245</v>
       </c>
       <c r="C102" s="1" t="s">
@@ -4890,7 +4890,7 @@
       <c r="A103" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B103" s="12" t="s">
+      <c r="B103" s="10" t="s">
         <v>240</v>
       </c>
       <c r="C103" s="1"/>
@@ -4902,7 +4902,7 @@
       <c r="A104" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B104" s="12" t="s">
+      <c r="B104" s="10" t="s">
         <v>248</v>
       </c>
       <c r="C104" s="1" t="s">
@@ -4922,7 +4922,7 @@
       <c r="A105" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B105" s="12" t="s">
+      <c r="B105" s="10" t="s">
         <v>251</v>
       </c>
       <c r="C105" s="1" t="s">
@@ -4937,7 +4937,7 @@
       <c r="A106" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B106" s="12" t="s">
+      <c r="B106" s="10" t="s">
         <v>254</v>
       </c>
       <c r="C106" s="1" t="s">
@@ -4952,7 +4952,7 @@
       <c r="A107" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B107" s="12" t="s">
+      <c r="B107" s="10" t="s">
         <v>248</v>
       </c>
       <c r="C107" s="1"/>
@@ -4965,10 +4965,12 @@
       <c r="B108" s="4" t="s">
         <v>257</v>
       </c>
-      <c r="C108" s="2"/>
+      <c r="C108" s="12" t="s">
+        <v>23</v>
+      </c>
       <c r="D108" s="2"/>
       <c r="E108" s="2"/>
-      <c r="F108" s="9" t="s">
+      <c r="F108" s="1" t="s">
         <v>258</v>
       </c>
       <c r="G108" s="2"/>
@@ -4999,7 +5001,9 @@
       <c r="B109" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="C109" s="1"/>
+      <c r="C109" s="13" t="s">
+        <v>23</v>
+      </c>
       <c r="D109" s="1"/>
       <c r="E109" s="1"/>
       <c r="F109" s="4"/>
@@ -5099,7 +5103,9 @@
       <c r="B112" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="C112" s="1"/>
+      <c r="C112" s="13" t="s">
+        <v>23</v>
+      </c>
       <c r="D112" s="14"/>
       <c r="E112" s="1"/>
       <c r="F112" s="1"/>
@@ -5233,7 +5239,9 @@
       <c r="B116" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="C116" s="1"/>
+      <c r="C116" s="13" t="s">
+        <v>23</v>
+      </c>
       <c r="D116" s="15"/>
       <c r="E116" s="1"/>
       <c r="F116" s="1"/>
@@ -5335,7 +5343,9 @@
       <c r="B119" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="C119" s="1"/>
+      <c r="C119" s="13" t="s">
+        <v>23</v>
+      </c>
       <c r="D119" s="15"/>
       <c r="E119" s="1"/>
       <c r="F119" s="1"/>
@@ -5471,7 +5481,9 @@
       <c r="B123" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="C123" s="1"/>
+      <c r="C123" s="13" t="s">
+        <v>23</v>
+      </c>
       <c r="D123" s="15"/>
       <c r="E123" s="1"/>
       <c r="F123" s="1" t="s">
@@ -5747,7 +5759,9 @@
       <c r="B131" s="1" t="s">
         <v>291</v>
       </c>
-      <c r="C131" s="1"/>
+      <c r="C131" s="13" t="s">
+        <v>23</v>
+      </c>
       <c r="D131" s="15"/>
       <c r="E131" s="1"/>
       <c r="F131" s="1" t="s">
@@ -5887,7 +5901,9 @@
       <c r="B135" s="1" t="s">
         <v>298</v>
       </c>
-      <c r="C135" s="1"/>
+      <c r="C135" s="13" t="s">
+        <v>23</v>
+      </c>
       <c r="D135" s="15"/>
       <c r="E135" s="1"/>
       <c r="F135" s="1" t="s">
@@ -6018,7 +6034,7 @@
       <c r="A139" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B139" s="12" t="s">
+      <c r="B139" s="10" t="s">
         <v>302</v>
       </c>
       <c r="C139" s="1" t="s">
@@ -6038,7 +6054,7 @@
       <c r="A140" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="B140" s="12" t="s">
+      <c r="B140" s="10" t="s">
         <v>306</v>
       </c>
       <c r="C140" s="1" t="s">
@@ -6056,7 +6072,7 @@
       <c r="A141" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="B141" s="12" t="s">
+      <c r="B141" s="10" t="s">
         <v>309</v>
       </c>
       <c r="C141" s="1" t="s">
@@ -6096,7 +6112,7 @@
       <c r="A142" s="1" t="s">
         <v>313</v>
       </c>
-      <c r="B142" s="12" t="s">
+      <c r="B142" s="10" t="s">
         <v>314</v>
       </c>
       <c r="C142" s="1" t="s">
@@ -6182,7 +6198,7 @@
       <c r="A144" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="B144" s="12" t="s">
+      <c r="B144" s="10" t="s">
         <v>326</v>
       </c>
       <c r="C144" s="1" t="s">
@@ -6200,7 +6216,7 @@
       <c r="A145" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B145" s="12" t="s">
+      <c r="B145" s="10" t="s">
         <v>302</v>
       </c>
       <c r="C145" s="1"/>
@@ -6211,7 +6227,7 @@
       <c r="A146" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B146" s="12" t="s">
+      <c r="B146" s="10" t="s">
         <v>329</v>
       </c>
       <c r="C146" s="1" t="s">
@@ -7754,7 +7770,7 @@
       <c r="A197" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B197" s="12" t="s">
+      <c r="B197" s="10" t="s">
         <v>470</v>
       </c>
       <c r="L197" s="1" t="s">
@@ -7765,7 +7781,7 @@
       <c r="A198" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B198" s="12" t="s">
+      <c r="B198" s="10" t="s">
         <v>472</v>
       </c>
       <c r="L198" s="1" t="s">
@@ -7776,7 +7792,7 @@
       <c r="A199" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B199" s="12" t="s">
+      <c r="B199" s="10" t="s">
         <v>474</v>
       </c>
       <c r="C199" s="4"/>
@@ -7810,7 +7826,7 @@
       <c r="A200" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B200" s="12" t="s">
+      <c r="B200" s="10" t="s">
         <v>476</v>
       </c>
       <c r="L200" s="1" t="s">
@@ -7820,49 +7836,49 @@
     <row r="201" ht="15.75" customHeight="1"/>
     <row r="202" ht="15.75" customHeight="1"/>
     <row r="203" ht="15.75" customHeight="1">
-      <c r="C203" s="12"/>
+      <c r="C203" s="10"/>
     </row>
     <row r="204" ht="15.75" customHeight="1">
-      <c r="B204" s="12"/>
-      <c r="C204" s="12"/>
+      <c r="B204" s="10"/>
+      <c r="C204" s="10"/>
     </row>
     <row r="205" ht="15.75" customHeight="1"/>
     <row r="206" ht="15.75" customHeight="1">
-      <c r="B206" s="12"/>
+      <c r="B206" s="10"/>
     </row>
     <row r="207" ht="15.75" customHeight="1">
       <c r="B207" s="1"/>
     </row>
     <row r="208" ht="15.75" customHeight="1">
-      <c r="B208" s="12"/>
+      <c r="B208" s="10"/>
     </row>
     <row r="209" ht="15.75" customHeight="1">
-      <c r="B209" s="12"/>
+      <c r="B209" s="10"/>
     </row>
     <row r="210" ht="15.75" customHeight="1">
       <c r="B210" s="1"/>
     </row>
     <row r="211" ht="15.75" customHeight="1">
-      <c r="B211" s="12"/>
+      <c r="B211" s="10"/>
     </row>
     <row r="212" ht="15.75" customHeight="1">
       <c r="B212" s="1"/>
     </row>
     <row r="213" ht="15.75" customHeight="1">
-      <c r="B213" s="12"/>
+      <c r="B213" s="10"/>
     </row>
     <row r="214" ht="15.75" customHeight="1">
       <c r="B214" s="1"/>
     </row>
     <row r="215" ht="15.75" customHeight="1">
-      <c r="B215" s="12"/>
+      <c r="B215" s="10"/>
     </row>
     <row r="216" ht="15.75" customHeight="1">
       <c r="B216" s="1"/>
     </row>
     <row r="217" ht="15.75" customHeight="1"/>
     <row r="218" ht="15.75" customHeight="1">
-      <c r="C218" s="12"/>
+      <c r="C218" s="10"/>
     </row>
     <row r="219" ht="15.75" customHeight="1">
       <c r="B219" s="1"/>
@@ -7872,10 +7888,10 @@
     </row>
     <row r="221" ht="15.75" customHeight="1"/>
     <row r="222" ht="15.75" customHeight="1">
-      <c r="B222" s="12"/>
+      <c r="B222" s="10"/>
     </row>
     <row r="223" ht="15.75" customHeight="1">
-      <c r="B223" s="12"/>
+      <c r="B223" s="10"/>
     </row>
     <row r="224" ht="15.75" customHeight="1"/>
     <row r="225" ht="15.75" customHeight="1"/>

</xml_diff>